<commit_message>
fix: corrige o bug de atualização do chrome para o scraping
</commit_message>
<xml_diff>
--- a/Estudos_de_python/nfe_00000000000000000000000000000000000000000000.xlsx
+++ b/Estudos_de_python/nfe_00000000000000000000000000000000000000000000.xlsx
@@ -413,17 +413,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="239" customWidth="1" min="8" max="8"/>
+    <col width="79" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -477,37 +477,222 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LA VICTORIE EAU DE PARFUM INTENSE 75ml</t>
+          <t>SIAGE MASC CAP ACELERA CRESC V3 250g</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>129.92</v>
+        <v>49.49</v>
       </c>
       <c r="D2" t="n">
-        <v>219.87</v>
+        <v>83.75</v>
       </c>
       <c r="E2" t="n">
-        <v>99.94</v>
+        <v>38.07</v>
       </c>
       <c r="F2" t="n">
-        <v>179.89</v>
+        <v>68.53</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7891033935482</t>
+          <t>7891033535064</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://res.cloudinary.com/beleza-na-web/image/upload/w_1500,f_auto,fl_progressive,q_auto:eco,w_1800,c_limit/e_trim/v1/imagens/product/E93548/0195f723-fa44-400b-86bf-960ccf2bbea9-intense-la-victorie-eudora-eau-de-parfum-feminino-75ml.png</t>
+          <t>https://m.media-amazon.com/images/I/41ADAhusy0L._AC_.jpg</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>SIAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SIAGE COND ACELERA CRESC V3 200ml</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>35.35</v>
+      </c>
+      <c r="D3" t="n">
+        <v>59.82</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27.19</v>
+      </c>
+      <c r="F3" t="n">
+        <v>48.94</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>7891033535019</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://down-br.img.susercontent.com/file/br-11134207-81z1k-mdys9f0b9pfma9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SIAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SIAGE COND LIS INT V3 200ml</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="n">
+        <v>33.94</v>
+      </c>
+      <c r="D4" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="E4" t="n">
+        <v>26.11</v>
+      </c>
+      <c r="F4" t="n">
+        <v>47</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>7891033535057</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/41qumjCtLnL._AC_SY300_SX300_QL70_ML2_.jpg</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SIAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SIAGE SHAMP LIS INT V3 250ml</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>31.81</v>
+      </c>
+      <c r="D5" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="E5" t="n">
+        <v>24.47</v>
+      </c>
+      <c r="F5" t="n">
+        <v>44.05</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>7891033535040</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/61RTx3xDWSL._AC_SL1500_.jpg</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SIAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SIAGE SHAMP ACELERA CRESC V3 250ml</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" t="n">
+        <v>33.94</v>
+      </c>
+      <c r="D6" t="n">
+        <v>57.44</v>
+      </c>
+      <c r="E6" t="n">
+        <v>26.11</v>
+      </c>
+      <c r="F6" t="n">
+        <v>47</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7891033535026</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://m.media-amazon.com/images/I/61t72BIfN6L.jpg</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>SIAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EUD MAKE PLT SOMBRAS TURBO 8g</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>44.11</v>
+      </c>
+      <c r="D7" t="n">
+        <v>74.65000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>33.93</v>
+      </c>
+      <c r="F7" t="n">
+        <v>61.07</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7891033899807</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://down-br.img.susercontent.com/file/br-11134207-7r98o-ma3gx2idutc29e</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>EUD</t>
         </is>
       </c>
     </row>

</xml_diff>